<commit_message>
feat(pca): workflow de aprovacao de demandas com motivo obrigatorio e rastreio de cortes
</commit_message>
<xml_diff>
--- a/data/catalogo_interno_2027.xlsx
+++ b/data/catalogo_interno_2027.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="678" documentId="11_11930A375271611AE2A2BB0A1210FB05C8E21255" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF8A7B7D-8E3F-4C75-BB60-A46086A0BDE4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D5A8166-2FD2-4B82-9D0E-E70380232A6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5281,8 +5281,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="6">
@@ -5318,7 +5317,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5348,6 +5347,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -5504,11 +5509,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6818,7 +6825,7 @@
       <c r="H37" s="23">
         <v>2027</v>
       </c>
-      <c r="I37" s="27">
+      <c r="I37" s="31">
         <v>13800</v>
       </c>
     </row>
@@ -6847,7 +6854,7 @@
       <c r="H38" s="23">
         <v>2027</v>
       </c>
-      <c r="I38" s="20">
+      <c r="I38" s="31">
         <v>190</v>
       </c>
     </row>
@@ -6876,7 +6883,7 @@
       <c r="H39" s="23">
         <v>2027</v>
       </c>
-      <c r="I39" s="27"/>
+      <c r="I39" s="31"/>
     </row>
     <row r="40" spans="1:9" ht="25.5">
       <c r="A40" s="6">
@@ -6903,11 +6910,11 @@
       <c r="H40" s="23">
         <v>2027</v>
       </c>
-      <c r="I40" s="27">
-        <v>3097.55</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="25.5">
+      <c r="I40" s="31">
+        <v>3502.88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="54.75" customHeight="1">
       <c r="A41" s="6">
         <v>71</v>
       </c>
@@ -6932,7 +6939,9 @@
       <c r="H41" s="23">
         <v>2027</v>
       </c>
-      <c r="I41" s="20"/>
+      <c r="I41" s="31">
+        <v>28.53</v>
+      </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="6">
@@ -6959,7 +6968,7 @@
       <c r="H42" s="23">
         <v>2027</v>
       </c>
-      <c r="I42" s="20">
+      <c r="I42" s="31">
         <v>1400</v>
       </c>
     </row>
@@ -6988,7 +6997,9 @@
       <c r="H43" s="23">
         <v>2027</v>
       </c>
-      <c r="I43" s="20"/>
+      <c r="I43" s="31">
+        <v>35</v>
+      </c>
     </row>
     <row r="44" spans="1:9" ht="25.5">
       <c r="A44" s="6">
@@ -7015,11 +7026,11 @@
       <c r="H44" s="23">
         <v>2027</v>
       </c>
-      <c r="I44" s="30">
+      <c r="I44" s="31">
         <v>8689.7199999999993</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="25.5">
+    <row r="45" spans="1:9" ht="24">
       <c r="A45" s="6">
         <v>78</v>
       </c>
@@ -7035,7 +7046,7 @@
       <c r="E45" s="15">
         <v>907</v>
       </c>
-      <c r="F45" s="6" t="s">
+      <c r="F45" s="32" t="s">
         <v>94</v>
       </c>
       <c r="G45" s="6" t="s">
@@ -7044,7 +7055,7 @@
       <c r="H45" s="23">
         <v>2027</v>
       </c>
-      <c r="I45" s="20"/>
+      <c r="I45" s="31"/>
     </row>
     <row r="46" spans="1:9" ht="25.5">
       <c r="A46" s="6">
@@ -7071,7 +7082,9 @@
       <c r="H46" s="23">
         <v>2027</v>
       </c>
-      <c r="I46" s="20"/>
+      <c r="I46" s="31">
+        <v>5400</v>
+      </c>
     </row>
     <row r="47" spans="1:9" ht="51" hidden="1">
       <c r="A47" s="6">
@@ -7233,7 +7246,7 @@
       <c r="H52" s="23">
         <v>2027</v>
       </c>
-      <c r="I52" s="20"/>
+      <c r="I52" s="31"/>
     </row>
     <row r="53" spans="1:9" ht="76.5">
       <c r="A53" s="6">
@@ -7260,7 +7273,7 @@
       <c r="H53" s="23">
         <v>2027</v>
       </c>
-      <c r="I53" s="20"/>
+      <c r="I53" s="31"/>
     </row>
     <row r="54" spans="1:9" ht="25.5">
       <c r="A54" s="6">
@@ -7287,7 +7300,7 @@
       <c r="H54" s="23">
         <v>2027</v>
       </c>
-      <c r="I54" s="20"/>
+      <c r="I54" s="31"/>
     </row>
     <row r="55" spans="1:9" ht="51" hidden="1">
       <c r="A55" s="6">
@@ -7341,7 +7354,7 @@
       <c r="H56" s="23">
         <v>2027</v>
       </c>
-      <c r="I56" s="20">
+      <c r="I56" s="31">
         <v>279</v>
       </c>
     </row>
@@ -7370,7 +7383,7 @@
       <c r="H57" s="23">
         <v>2027</v>
       </c>
-      <c r="I57" s="20">
+      <c r="I57" s="31">
         <v>185</v>
       </c>
     </row>
@@ -7399,7 +7412,7 @@
       <c r="H58" s="23">
         <v>2027</v>
       </c>
-      <c r="I58" s="30">
+      <c r="I58" s="31">
         <v>264</v>
       </c>
     </row>
@@ -7428,7 +7441,7 @@
       <c r="H59" s="23">
         <v>2027</v>
       </c>
-      <c r="I59" s="20"/>
+      <c r="I59" s="31"/>
     </row>
     <row r="60" spans="1:9" ht="25.5" hidden="1">
       <c r="A60" s="6">
@@ -7482,7 +7495,7 @@
       <c r="H61" s="23">
         <v>2027</v>
       </c>
-      <c r="I61" s="20">
+      <c r="I61" s="31">
         <v>847</v>
       </c>
     </row>
@@ -7511,7 +7524,7 @@
       <c r="H62" s="23">
         <v>2027</v>
       </c>
-      <c r="I62" s="20"/>
+      <c r="I62" s="31"/>
     </row>
     <row r="63" spans="1:9">
       <c r="A63" s="6">
@@ -7538,7 +7551,7 @@
       <c r="H63" s="23">
         <v>2027</v>
       </c>
-      <c r="I63" s="27">
+      <c r="I63" s="31">
         <v>4260.5600000000004</v>
       </c>
     </row>
@@ -7567,7 +7580,7 @@
       <c r="H64" s="23">
         <v>2027</v>
       </c>
-      <c r="I64" s="20"/>
+      <c r="I64" s="31"/>
     </row>
     <row r="65" spans="1:9">
       <c r="A65" s="6">
@@ -7594,7 +7607,7 @@
       <c r="H65" s="23">
         <v>2027</v>
       </c>
-      <c r="I65" s="20">
+      <c r="I65" s="31">
         <v>200</v>
       </c>
     </row>
@@ -7623,7 +7636,7 @@
       <c r="H66" s="23">
         <v>2027</v>
       </c>
-      <c r="I66" s="20">
+      <c r="I66" s="31">
         <v>84</v>
       </c>
     </row>
@@ -7652,7 +7665,7 @@
       <c r="H67" s="23">
         <v>2027</v>
       </c>
-      <c r="I67" s="20">
+      <c r="I67" s="31">
         <v>105.24</v>
       </c>
     </row>
@@ -7681,7 +7694,7 @@
       <c r="H68" s="23">
         <v>2027</v>
       </c>
-      <c r="I68" s="20"/>
+      <c r="I68" s="31"/>
     </row>
     <row r="69" spans="1:9" ht="25.5">
       <c r="A69" s="6">
@@ -7708,7 +7721,7 @@
       <c r="H69" s="23">
         <v>2027</v>
       </c>
-      <c r="I69" s="20">
+      <c r="I69" s="31">
         <v>804</v>
       </c>
     </row>
@@ -7737,7 +7750,7 @@
       <c r="H70" s="23">
         <v>2027</v>
       </c>
-      <c r="I70" s="20"/>
+      <c r="I70" s="31"/>
     </row>
     <row r="71" spans="1:9" ht="63.75">
       <c r="A71" s="6">
@@ -7764,7 +7777,7 @@
       <c r="H71" s="23">
         <v>2027</v>
       </c>
-      <c r="I71" s="20"/>
+      <c r="I71" s="31"/>
     </row>
     <row r="72" spans="1:9" ht="25.5">
       <c r="A72" s="6">
@@ -7791,7 +7804,7 @@
       <c r="H72" s="23">
         <v>2027</v>
       </c>
-      <c r="I72" s="20"/>
+      <c r="I72" s="31"/>
     </row>
     <row r="73" spans="1:9" ht="25.5">
       <c r="A73" s="6">
@@ -7818,7 +7831,7 @@
       <c r="H73" s="23">
         <v>2027</v>
       </c>
-      <c r="I73" s="20"/>
+      <c r="I73" s="31"/>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" s="6">
@@ -7845,7 +7858,7 @@
       <c r="H74" s="23">
         <v>2027</v>
       </c>
-      <c r="I74" s="20">
+      <c r="I74" s="31">
         <v>98.44</v>
       </c>
     </row>
@@ -7874,7 +7887,7 @@
       <c r="H75" s="23">
         <v>2027</v>
       </c>
-      <c r="I75" s="20"/>
+      <c r="I75" s="31"/>
     </row>
     <row r="76" spans="1:9" ht="25.5">
       <c r="A76" s="6">
@@ -7901,7 +7914,7 @@
       <c r="H76" s="23">
         <v>2027</v>
       </c>
-      <c r="I76" s="30">
+      <c r="I76" s="31">
         <v>635.38</v>
       </c>
     </row>
@@ -7930,7 +7943,7 @@
       <c r="H77" s="23">
         <v>2027</v>
       </c>
-      <c r="I77" s="20"/>
+      <c r="I77" s="31"/>
     </row>
     <row r="78" spans="1:9" ht="25.5">
       <c r="A78" s="6">
@@ -7957,7 +7970,7 @@
       <c r="H78" s="23">
         <v>2027</v>
       </c>
-      <c r="I78" s="20"/>
+      <c r="I78" s="31"/>
     </row>
     <row r="79" spans="1:9" ht="25.5">
       <c r="A79" s="6">
@@ -7984,7 +7997,7 @@
       <c r="H79" s="23">
         <v>2027</v>
       </c>
-      <c r="I79" s="20"/>
+      <c r="I79" s="31"/>
     </row>
     <row r="80" spans="1:9" ht="25.5">
       <c r="A80" s="6">
@@ -8011,7 +8024,7 @@
       <c r="H80" s="23">
         <v>2027</v>
       </c>
-      <c r="I80" s="20"/>
+      <c r="I80" s="31"/>
     </row>
     <row r="81" spans="1:9" ht="25.5">
       <c r="A81" s="6">
@@ -8038,7 +8051,7 @@
       <c r="H81" s="23">
         <v>2027</v>
       </c>
-      <c r="I81" s="20"/>
+      <c r="I81" s="31"/>
     </row>
     <row r="82" spans="1:9" ht="25.5">
       <c r="A82" s="6">
@@ -8065,7 +8078,7 @@
       <c r="H82" s="23">
         <v>2027</v>
       </c>
-      <c r="I82" s="20"/>
+      <c r="I82" s="31"/>
     </row>
     <row r="83" spans="1:9" ht="25.5">
       <c r="A83" s="6">
@@ -8092,7 +8105,7 @@
       <c r="H83" s="23">
         <v>2027</v>
       </c>
-      <c r="I83" s="20"/>
+      <c r="I83" s="31"/>
     </row>
     <row r="84" spans="1:9" ht="25.5">
       <c r="A84" s="6">
@@ -8119,7 +8132,7 @@
       <c r="H84" s="23">
         <v>2027</v>
       </c>
-      <c r="I84" s="20"/>
+      <c r="I84" s="31"/>
     </row>
     <row r="85" spans="1:9" ht="25.5">
       <c r="A85" s="6">
@@ -8146,7 +8159,7 @@
       <c r="H85" s="23">
         <v>2027</v>
       </c>
-      <c r="I85" s="20"/>
+      <c r="I85" s="31"/>
     </row>
     <row r="86" spans="1:9">
       <c r="A86" s="6">
@@ -8173,7 +8186,7 @@
       <c r="H86" s="23">
         <v>2027</v>
       </c>
-      <c r="I86" s="27">
+      <c r="I86" s="31">
         <v>13067.16</v>
       </c>
     </row>
@@ -8202,7 +8215,7 @@
       <c r="H87" s="23">
         <v>2027</v>
       </c>
-      <c r="I87" s="27">
+      <c r="I87" s="31">
         <v>19305.55</v>
       </c>
     </row>
@@ -8231,7 +8244,7 @@
       <c r="H88" s="23">
         <v>2027</v>
       </c>
-      <c r="I88" s="20"/>
+      <c r="I88" s="31"/>
     </row>
     <row r="89" spans="1:9" ht="25.5">
       <c r="A89" s="6">
@@ -8258,7 +8271,7 @@
       <c r="H89" s="23">
         <v>2027</v>
       </c>
-      <c r="I89" s="20"/>
+      <c r="I89" s="31"/>
     </row>
     <row r="90" spans="1:9" ht="38.25" hidden="1">
       <c r="A90" s="6">
@@ -8453,7 +8466,7 @@
       <c r="H96" s="23">
         <v>2027</v>
       </c>
-      <c r="I96" s="20"/>
+      <c r="I96" s="31"/>
     </row>
     <row r="97" spans="1:9" ht="89.25" hidden="1">
       <c r="A97" s="6">
@@ -8710,7 +8723,7 @@
       <c r="H105" s="23">
         <v>2027</v>
       </c>
-      <c r="I105" s="20"/>
+      <c r="I105" s="31"/>
     </row>
     <row r="106" spans="1:9">
       <c r="A106" s="6">
@@ -8737,7 +8750,7 @@
       <c r="H106" s="23">
         <v>2027</v>
       </c>
-      <c r="I106" s="27">
+      <c r="I106" s="31">
         <v>1056600</v>
       </c>
     </row>
@@ -8766,7 +8779,7 @@
       <c r="H107" s="23">
         <v>2027</v>
       </c>
-      <c r="I107" s="27">
+      <c r="I107" s="31">
         <v>77183.649999999994</v>
       </c>
     </row>
@@ -8795,7 +8808,7 @@
       <c r="H108" s="23">
         <v>2027</v>
       </c>
-      <c r="I108" s="20"/>
+      <c r="I108" s="31"/>
     </row>
     <row r="109" spans="1:9">
       <c r="A109" s="6">
@@ -8822,7 +8835,7 @@
       <c r="H109" s="23">
         <v>2027</v>
       </c>
-      <c r="I109" s="20"/>
+      <c r="I109" s="31"/>
     </row>
     <row r="110" spans="1:9">
       <c r="A110" s="6">
@@ -8849,7 +8862,7 @@
       <c r="H110" s="23">
         <v>2027</v>
       </c>
-      <c r="I110" s="20"/>
+      <c r="I110" s="31"/>
     </row>
     <row r="111" spans="1:9">
       <c r="A111" s="6">
@@ -8876,7 +8889,7 @@
       <c r="H111" s="23">
         <v>2027</v>
       </c>
-      <c r="I111" s="20"/>
+      <c r="I111" s="31"/>
     </row>
     <row r="112" spans="1:9">
       <c r="A112" s="6">
@@ -8903,7 +8916,7 @@
       <c r="H112" s="23">
         <v>2027</v>
       </c>
-      <c r="I112" s="20"/>
+      <c r="I112" s="31"/>
     </row>
     <row r="113" spans="1:9">
       <c r="A113" s="6">
@@ -8930,7 +8943,7 @@
       <c r="H113" s="23">
         <v>2027</v>
       </c>
-      <c r="I113" s="20"/>
+      <c r="I113" s="31"/>
     </row>
     <row r="114" spans="1:9">
       <c r="A114" s="6">
@@ -8957,7 +8970,7 @@
       <c r="H114" s="23">
         <v>2027</v>
       </c>
-      <c r="I114" s="20"/>
+      <c r="I114" s="31"/>
     </row>
     <row r="115" spans="1:9">
       <c r="A115" s="6">
@@ -8984,7 +8997,7 @@
       <c r="H115" s="23">
         <v>2027</v>
       </c>
-      <c r="I115" s="20"/>
+      <c r="I115" s="31"/>
     </row>
     <row r="116" spans="1:9">
       <c r="A116" s="6">
@@ -9011,7 +9024,7 @@
       <c r="H116" s="23">
         <v>2027</v>
       </c>
-      <c r="I116" s="20"/>
+      <c r="I116" s="31"/>
     </row>
     <row r="117" spans="1:9">
       <c r="A117" s="6">
@@ -9038,7 +9051,7 @@
       <c r="H117" s="23">
         <v>2027</v>
       </c>
-      <c r="I117" s="20"/>
+      <c r="I117" s="31"/>
     </row>
     <row r="118" spans="1:9">
       <c r="A118" s="6">
@@ -9065,7 +9078,7 @@
       <c r="H118" s="23">
         <v>2027</v>
       </c>
-      <c r="I118" s="20"/>
+      <c r="I118" s="31"/>
     </row>
     <row r="119" spans="1:9" ht="25.5">
       <c r="A119" s="6">
@@ -9092,7 +9105,7 @@
       <c r="H119" s="23">
         <v>2027</v>
       </c>
-      <c r="I119" s="20">
+      <c r="I119" s="31">
         <v>408</v>
       </c>
     </row>
@@ -9148,7 +9161,7 @@
       <c r="H121" s="23">
         <v>2027</v>
       </c>
-      <c r="I121" s="20"/>
+      <c r="I121" s="31"/>
     </row>
     <row r="122" spans="1:9" ht="63.75" hidden="1">
       <c r="A122" s="6">
@@ -9867,7 +9880,7 @@
       <c r="H146" s="23">
         <v>2027</v>
       </c>
-      <c r="I146" s="31">
+      <c r="I146" s="30">
         <v>38.35</v>
       </c>
     </row>
@@ -11002,7 +11015,7 @@
       <c r="H187" s="23">
         <v>2027</v>
       </c>
-      <c r="I187" s="20"/>
+      <c r="I187" s="31"/>
     </row>
     <row r="188" spans="1:9" ht="38.25" hidden="1">
       <c r="A188" s="6">
@@ -11286,7 +11299,7 @@
       <c r="H197" s="23">
         <v>2027</v>
       </c>
-      <c r="I197" s="20">
+      <c r="I197" s="31">
         <v>456</v>
       </c>
     </row>
@@ -12706,7 +12719,7 @@
       <c r="H247" s="23">
         <v>2027</v>
       </c>
-      <c r="I247" s="20">
+      <c r="I247" s="31">
         <v>577.83000000000004</v>
       </c>
     </row>
@@ -12735,7 +12748,7 @@
       <c r="H248" s="23">
         <v>2027</v>
       </c>
-      <c r="I248" s="32">
+      <c r="I248" s="31">
         <v>20980</v>
       </c>
     </row>
@@ -12791,7 +12804,7 @@
       <c r="H250" s="23">
         <v>2027</v>
       </c>
-      <c r="I250" s="20"/>
+      <c r="I250" s="31"/>
     </row>
     <row r="251" spans="1:9" ht="51" hidden="1">
       <c r="A251" s="6">
@@ -13108,7 +13121,7 @@
       <c r="H261" s="23">
         <v>2027</v>
       </c>
-      <c r="I261" s="20"/>
+      <c r="I261" s="31"/>
     </row>
     <row r="262" spans="1:9" ht="38.25" hidden="1">
       <c r="A262" s="6">
@@ -13390,7 +13403,7 @@
       <c r="H271" s="23">
         <v>2027</v>
       </c>
-      <c r="I271" s="20">
+      <c r="I271" s="31">
         <v>204.88</v>
       </c>
     </row>
@@ -13529,7 +13542,7 @@
       <c r="H276" s="23">
         <v>2027</v>
       </c>
-      <c r="I276" s="27">
+      <c r="I276" s="31">
         <v>1614.2</v>
       </c>
     </row>
@@ -13755,7 +13768,7 @@
       <c r="H284" s="23">
         <v>2027</v>
       </c>
-      <c r="I284" s="20">
+      <c r="I284" s="31">
         <v>671</v>
       </c>
     </row>
@@ -13784,7 +13797,7 @@
       <c r="H285" s="23">
         <v>2027</v>
       </c>
-      <c r="I285" s="20">
+      <c r="I285" s="31">
         <v>526</v>
       </c>
     </row>
@@ -14635,7 +14648,7 @@
       <c r="H316" s="23">
         <v>2027</v>
       </c>
-      <c r="I316" s="20"/>
+      <c r="I316" s="31"/>
     </row>
     <row r="317" spans="1:9" ht="25.5" hidden="1">
       <c r="A317" s="6">
@@ -14878,7 +14891,7 @@
       <c r="H325" s="23">
         <v>2027</v>
       </c>
-      <c r="I325" s="20"/>
+      <c r="I325" s="31"/>
     </row>
     <row r="326" spans="1:9" ht="24" hidden="1">
       <c r="A326" s="6">

</xml_diff>